<commit_message>
Atualiza base_aderencia (22/09/2026 09:27)
</commit_message>
<xml_diff>
--- a/base_aderencia.xlsx
+++ b/base_aderencia.xlsx
@@ -530,7 +530,7 @@
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>67486</v>
+        <v>67134</v>
       </c>
       <c r="M2" t="n">
         <v>1</v>
@@ -583,10 +583,10 @@
         <v>100005</v>
       </c>
       <c r="L3" t="n">
-        <v>78156</v>
+        <v>95932</v>
       </c>
       <c r="M3" t="n">
-        <v>0.7815209239538023</v>
+        <v>0.95927203639818</v>
       </c>
     </row>
     <row r="4">
@@ -907,10 +907,10 @@
         <v>35033</v>
       </c>
       <c r="L9" t="n">
-        <v>12321</v>
+        <v>28227</v>
       </c>
       <c r="M9" t="n">
-        <v>0.3516969714269403</v>
+        <v>0.8057260297433848</v>
       </c>
     </row>
     <row r="10">
@@ -3813,10 +3813,10 @@
         <v>0</v>
       </c>
       <c r="L63" t="n">
-        <v>0</v>
+        <v>2378</v>
       </c>
       <c r="M63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -4938,10 +4938,10 @@
         <v>175509</v>
       </c>
       <c r="L84" t="n">
-        <v>327691</v>
+        <v>352859</v>
       </c>
       <c r="M84" t="n">
-        <v>1.867089437008928</v>
+        <v>2.010489490567435</v>
       </c>
     </row>
     <row r="85">
@@ -6193,10 +6193,10 @@
         <v>1086.5</v>
       </c>
       <c r="L107" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="M107" t="n">
-        <v>0</v>
+        <v>1.104463874827428</v>
       </c>
     </row>
     <row r="108">
@@ -6248,10 +6248,10 @@
         <v>957</v>
       </c>
       <c r="L108" t="n">
-        <v>257</v>
+        <v>2353</v>
       </c>
       <c r="M108" t="n">
-        <v>0.2685475444096134</v>
+        <v>2.458725182863114</v>
       </c>
     </row>
     <row r="109">
@@ -6576,10 +6576,10 @@
         <v>31247.83334</v>
       </c>
       <c r="L114" t="n">
-        <v>27722</v>
+        <v>31772</v>
       </c>
       <c r="M114" t="n">
-        <v>0.8871655099527613</v>
+        <v>1.016774496148154</v>
       </c>
     </row>
     <row r="115">
@@ -6841,10 +6841,10 @@
         <v>7091.833339999999</v>
       </c>
       <c r="L119" t="n">
-        <v>8798</v>
+        <v>18615</v>
       </c>
       <c r="M119" t="n">
-        <v>1.240581888801126</v>
+        <v>2.624850177316773</v>
       </c>
     </row>
     <row r="120">
@@ -6947,10 +6947,10 @@
         <v>16157.00001</v>
       </c>
       <c r="L121" t="n">
-        <v>10054</v>
+        <v>17905</v>
       </c>
       <c r="M121" t="n">
-        <v>0.6222689851938671</v>
+        <v>1.108188400626237</v>
       </c>
     </row>
     <row r="122">
@@ -9385,7 +9385,7 @@
         <v>0</v>
       </c>
       <c r="L167" t="n">
-        <v>3861</v>
+        <v>3896</v>
       </c>
       <c r="M167" t="n">
         <v>1</v>
@@ -9650,10 +9650,10 @@
         <v>0</v>
       </c>
       <c r="L172" t="n">
-        <v>0</v>
+        <v>2303</v>
       </c>
       <c r="M172" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="173">

</xml_diff>

<commit_message>
Atualiza base_aderencia (22/09/2026 09:38)
</commit_message>
<xml_diff>
--- a/base_aderencia.xlsx
+++ b/base_aderencia.xlsx
@@ -5240,7 +5240,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>2LT</t>
+          <t>2L</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -5295,7 +5295,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>2LT</t>
+          <t>2L</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -5350,7 +5350,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>2LT</t>
+          <t>2L</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -5405,7 +5405,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>2LT</t>
+          <t>2L</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -5460,7 +5460,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>2LT</t>
+          <t>2L</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -5515,7 +5515,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>2LT</t>
+          <t>2L</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -5570,7 +5570,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>2LT</t>
+          <t>2L</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -5625,7 +5625,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>2LT</t>
+          <t>2L</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -5680,7 +5680,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>2LT</t>
+          <t>2L</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
@@ -5735,7 +5735,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>2LT</t>
+          <t>2L</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -5790,7 +5790,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>2LT</t>
+          <t>2L</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -5845,7 +5845,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>2LT</t>
+          <t>2L</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -5900,7 +5900,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>2LT</t>
+          <t>2L</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
@@ -5955,7 +5955,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>2LT</t>
+          <t>2L</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -6010,7 +6010,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>2LT</t>
+          <t>2L</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
@@ -6065,7 +6065,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>2LT</t>
+          <t>2L</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
@@ -6120,7 +6120,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>2LT</t>
+          <t>2L</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
@@ -6340,7 +6340,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>2,5LT</t>
+          <t>2,5L</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
@@ -6395,7 +6395,7 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>2,5LT</t>
+          <t>2,5L</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
@@ -6450,7 +6450,7 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>2,5LT</t>
+          <t>2,5L</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">

</xml_diff>